<commit_message>
add and fix documents
</commit_message>
<xml_diff>
--- a/docs/DB詳細設計書.xlsx
+++ b/docs/DB詳細設計書.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\source\repos2\shopping-sight\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D1EDE09-8AF2-4ACE-94AB-683693B3DB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82308DB-D385-4332-8F04-4D0B0BC89A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C6D2EF96-38BB-443A-A710-98225FDEE50F}"/>
+    <workbookView xWindow="19710" yWindow="0" windowWidth="15830" windowHeight="10170" firstSheet="3" activeTab="8" xr2:uid="{C6D2EF96-38BB-443A-A710-98225FDEE50F}"/>
   </bookViews>
   <sheets>
-    <sheet name="商品" sheetId="1" r:id="rId1"/>
-    <sheet name="商品画像" sheetId="2" r:id="rId2"/>
-    <sheet name="カテゴリー" sheetId="3" r:id="rId3"/>
-    <sheet name="ユーザー" sheetId="4" r:id="rId4"/>
+    <sheet name="ユーザー" sheetId="4" r:id="rId1"/>
+    <sheet name="カテゴリー" sheetId="3" r:id="rId2"/>
+    <sheet name="商品" sheetId="1" r:id="rId3"/>
+    <sheet name="商品画像" sheetId="2" r:id="rId4"/>
     <sheet name="カート" sheetId="5" r:id="rId5"/>
-    <sheet name="注文" sheetId="6" r:id="rId6"/>
-    <sheet name="注文明細" sheetId="7" r:id="rId7"/>
-    <sheet name="管理者" sheetId="8" r:id="rId8"/>
+    <sheet name="管理者" sheetId="8" r:id="rId6"/>
+    <sheet name="注文" sheetId="6" r:id="rId7"/>
+    <sheet name="注文明細" sheetId="7" r:id="rId8"/>
+    <sheet name="在庫" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,8 +35,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -46,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="130">
   <si>
     <t>No</t>
   </si>
@@ -291,18 +290,12 @@
     <t xml:space="preserve"> 合計金額 </t>
   </si>
   <si>
-    <t xml:space="preserve"> delivery_method </t>
-  </si>
-  <si>
     <t xml:space="preserve"> VARCHAR(20) </t>
   </si>
   <si>
     <t xml:space="preserve"> 置き配/対面 </t>
   </si>
   <si>
-    <t xml:space="preserve"> stripe_payment_intent_id </t>
-  </si>
-  <si>
     <t xml:space="preserve"> VARCHAR(255) </t>
   </si>
   <si>
@@ -388,6 +381,123 @@
   </si>
   <si>
     <t>権限（0:一般 / 1:上位）</t>
+  </si>
+  <si>
+    <t>status</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>INT</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ステータス</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>〇</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">payment_method </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>payment_id</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>■在庫履歴</t>
+    <rPh sb="1" eb="3">
+      <t>ザイコ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>リレキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>履歴ID</t>
+    <rPh sb="0" eb="2">
+      <t>リレキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>商品ID</t>
+    <rPh sb="0" eb="2">
+      <t>ショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者ID</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>在庫増減</t>
+    <rPh sb="0" eb="2">
+      <t>ザイコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ゾウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>説明</t>
+    <rPh sb="0" eb="2">
+      <t>セツメイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>在庫変更時の日時</t>
+    <rPh sb="0" eb="4">
+      <t>ザイコヘンコウ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ジ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ニチジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> INT </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> product_id</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> admin_id</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> change</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> note</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> created_at</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> VARCHAR(255)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -814,25 +924,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21B289EE-9BED-437F-8EDB-D9C52F9C3FDB}">
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5978DB-A54C-48C3-8FAE-32A78C147FB6}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="4.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.08203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.58203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -846,19 +956,16 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -871,18 +978,17 @@
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -890,212 +996,108 @@
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G5" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G6" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F8" s="2"/>
+      <c r="G8" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="1">
-        <v>10</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="1">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="1">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1105,24 +1107,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41BA15DC-FF21-4E95-ABD8-B90613FFBD26}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A678F37C-A2AA-42D0-9305-E73B922A2BBE}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="4.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.08203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1136,16 +1138,13 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1158,55 +1157,50 @@
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="F3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>42</v>
+        <v>109</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>110</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="F5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1218,8 +1212,7 @@
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1230,24 +1223,25 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A678F37C-A2AA-42D0-9305-E73B922A2BBE}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21B289EE-9BED-437F-8EDB-D9C52F9C3FDB}">
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.08203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.58203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1261,13 +1255,19 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1280,14 +1280,18 @@
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -1295,22 +1299,24 @@
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
@@ -1318,7 +1324,187 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>45</v>
+        <v>10</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="1">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="1">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="1">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1328,25 +1514,24 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5978DB-A54C-48C3-8FAE-32A78C147FB6}">
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41BA15DC-FF21-4E95-ABD8-B90613FFBD26}">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1360,16 +1545,16 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1382,126 +1567,69 @@
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="G4" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1513,22 +1641,22 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91AC3966-E88E-4086-B132-B69CE8A90EDD}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.58203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1548,7 +1676,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1568,7 +1696,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -1586,7 +1714,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1604,7 +1732,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1622,7 +1750,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1647,219 +1775,146 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61ABE213-E731-4FA5-85AC-10FC6030CD77}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA2D541C-1367-43A8-AA68-C742DC52CB88}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="8.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.58203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A2" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="H2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3" s="4">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="4">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A5" s="4">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A6" s="4">
+      <c r="E2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="H6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A7" s="4">
+      <c r="B6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8" s="4">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A9" s="4">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>89</v>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1869,48 +1924,52 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{095F035D-56CF-45A8-91B6-AF7DB8CB7FED}">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61ABE213-E731-4FA5-85AC-10FC6030CD77}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.08203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1930,15 +1989,18 @@
         <v>73</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+        <v>74</v>
+      </c>
+      <c r="H3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>72</v>
@@ -1953,15 +2015,18 @@
         <v>73</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+        <v>76</v>
+      </c>
+      <c r="H4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>72</v>
@@ -1970,24 +2035,24 @@
         <v>70</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>73</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>70</v>
@@ -1999,18 +2064,21 @@
         <v>73</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+        <v>80</v>
+      </c>
+      <c r="H6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>70</v>
@@ -2018,11 +2086,55 @@
       <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="4"/>
+      <c r="G7" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>106</v>
+      <c r="G8" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2032,146 +2144,344 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA2D541C-1367-43A8-AA68-C742DC52CB88}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{095F035D-56CF-45A8-91B6-AF7DB8CB7FED}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B3" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B4" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="B5" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="B7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96B3DD6B-FBC4-4BC1-89DC-932C248B5BB4}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="10.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.08203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="1">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2" t="s">
-        <v>37</v>
+      <c r="B8" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>